<commit_message>
Create Sprint: sprint number as text with leading zeros
The sprint number is now a text box, and {number} in sprint names and
goals is written with at least two digits (1 -> 01). Extra digits typed
are kept (001), and the next number keeps the same width (09 -> 10).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199WRKsVKq4eroZLJmPLsXK
</commit_message>
<xml_diff>
--- a/config/sprints.xlsx
+++ b/config/sprints.xlsx
@@ -665,7 +665,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Optional. Placeholders: {team}, {project}, {number}. Default: {team} Sprint {number}</t>
+          <t>Optional. Placeholders: {team}, {project}, {number}. Default: {team} Sprint {number}. {number} is written with at least 2 digits: 01, 02 ... 10.</t>
         </is>
       </c>
     </row>
@@ -689,7 +689,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>That sprint's start date. Later sprints follow on back to back, one sprint length apart.</t>
+          <t>That sprint's start date, as an Excel date or text like 2026-01-05. Later sprints follow on back to back, one sprint length apart.</t>
         </is>
       </c>
     </row>

</xml_diff>